<commit_message>
feat: extended MS scoring comparison — 15 variants benchmarked
Add 6 new scoring methods to ms_scoring.py: warm weight rescaling,
squared Z-Score, TF-IDF ingredient weighting, top-K scoring, cosine
similarity, and ensemble averaging. Notebook section 17 runs all 15
combinations and ranks by accuracy. Z-Score (60%) remains best MS
variant; cosine similarity underperforms due to the sparse weight matrix.
</commit_message>
<xml_diff>
--- a/outputs/scoring_ms_assessment.xlsx
+++ b/outputs/scoring_ms_assessment.xlsx
@@ -16,6 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MS_Scores_ZScore" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MS_Assignments_All" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation_vs_Melanie" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended_Method_Comparison" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best_MS_Assignments" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4123,6 +4125,2723 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy_%</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>warm_n</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>green_n</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Unpl_n</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>other_n</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MS Z-Score</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E2" t="n">
+        <v>69</v>
+      </c>
+      <c r="F2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ensemble orig+Z</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E3" t="n">
+        <v>85</v>
+      </c>
+      <c r="F3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MS original</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" t="n">
+        <v>88</v>
+      </c>
+      <c r="F4" t="n">
+        <v>26</v>
+      </c>
+      <c r="G4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Warm rescale</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>50</v>
+      </c>
+      <c r="E5" t="n">
+        <v>62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44</v>
+      </c>
+      <c r="G5" t="n">
+        <v>22</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Warm + Z-Score</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="n">
+        <v>41</v>
+      </c>
+      <c r="F6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G6" t="n">
+        <v>28</v>
+      </c>
+      <c r="H6" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TF-IDF</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="n">
+        <v>92</v>
+      </c>
+      <c r="F7" t="n">
+        <v>21</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TF-IDF + warm</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" t="n">
+        <v>68</v>
+      </c>
+      <c r="F8" t="n">
+        <v>36</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Top-5</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" t="n">
+        <v>91</v>
+      </c>
+      <c r="F9" t="n">
+        <v>22</v>
+      </c>
+      <c r="G9" t="n">
+        <v>15</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Top-5 + warm</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" t="n">
+        <v>66</v>
+      </c>
+      <c r="F10" t="n">
+        <v>39</v>
+      </c>
+      <c r="G10" t="n">
+        <v>21</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ensemble warm+Z</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>50</v>
+      </c>
+      <c r="E11" t="n">
+        <v>58</v>
+      </c>
+      <c r="F11" t="n">
+        <v>37</v>
+      </c>
+      <c r="G11" t="n">
+        <v>26</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MS Rohstoffe</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" t="n">
+        <v>35</v>
+      </c>
+      <c r="F12" t="n">
+        <v>79</v>
+      </c>
+      <c r="G12" t="n">
+        <v>16</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Squared Z-Score</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" t="n">
+        <v>40</v>
+      </c>
+      <c r="E13" t="n">
+        <v>61</v>
+      </c>
+      <c r="F13" t="n">
+        <v>31</v>
+      </c>
+      <c r="G13" t="n">
+        <v>19</v>
+      </c>
+      <c r="H13" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Warm + Sq.Z-Score</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="n">
+        <v>37</v>
+      </c>
+      <c r="F14" t="n">
+        <v>44</v>
+      </c>
+      <c r="G14" t="n">
+        <v>26</v>
+      </c>
+      <c r="H14" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cosine</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" t="n">
+        <v>20</v>
+      </c>
+      <c r="E15" t="n">
+        <v>54</v>
+      </c>
+      <c r="F15" t="n">
+        <v>60</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cosine + warm</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" t="n">
+        <v>54</v>
+      </c>
+      <c r="F16" t="n">
+        <v>60</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C131"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rez.-Nr.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MS_cluster</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>panel_cluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>185.028</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>185.043P</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>185.044</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>185.046</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>185.086</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>185.090P</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>185.091</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>185.133</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>185.178HP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>185.237H</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>185.239</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>185.267</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>185.291</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>185.294</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>185.309P</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>185.314</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>185.321</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>185.339P</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>185.382P</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>185.471</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>185.507P</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>185.513P</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>185.514</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>185.578P</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>185.615</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>185.621P</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>185.644P</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>185.664</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>185.675P</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>185.727P</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>185.741P</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>185.748P</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>185.796P</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>185.902P</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>185.922P</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>185.984P</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>186.179P</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>186.190P</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>186.192</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>186.277P</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>186.293P</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>186.395P</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>186.396P</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>186.490P</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>186.569P</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>186.821</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>186.950P</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>186.981P</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>186.985P</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>187.004P</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>187.015P</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>187.061P</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>187.064P</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>187.119P</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>187.167P</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>187.246P</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>187.365</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>187.414P</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>exotic</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>187.482P</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>187.483P</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>187.507P</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>187.519P</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>187.521P</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>187.522P</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>187.567P</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>187.571P</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>187.608P</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>187.657P</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>187.662P</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t>187.694P</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>187.695P</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>187.746P</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>187.752P</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t>187.753P</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>187.772</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>exotic</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>187.773P</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>187.776</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>187.783P</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>187.786P</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>187.787P</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>187.791P</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>187.796P</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>187.799P</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>187.800P</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="inlineStr">
+        <is>
+          <t>187.826P</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>187.829P</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
+        <is>
+          <t>187.834P</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="inlineStr">
+        <is>
+          <t>187.843P</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>187.870P</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>187.871P</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>187.885P</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>187.886P</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>187.892P</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>187.893P</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>187.894P</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>187.895P</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>187.896P</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr">
+        <is>
+          <t>187.897P</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>187.907</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>187.914P</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>187.916P</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>187.920P</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>187.921P</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>187.923P</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>188.118P</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>188.375P</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr">
+        <is>
+          <t>188.402P</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
+          <t>188.412P</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
+        <is>
+          <t>188.462KHP</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>188.481KHP</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
+        <is>
+          <t>188.491P</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="inlineStr">
+        <is>
+          <t>188.560P</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="inlineStr">
+        <is>
+          <t>188.628P</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="inlineStr">
+        <is>
+          <t>188.639P</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="inlineStr">
+        <is>
+          <t>188.656P</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="inlineStr">
+        <is>
+          <t>188.668P</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="inlineStr">
+        <is>
+          <t>188.740P</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="inlineStr">
+        <is>
+          <t>188.819</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>188.820</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
+          <t>188.822</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="inlineStr">
+        <is>
+          <t>188.866</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="inlineStr">
+        <is>
+          <t>188.894</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="inlineStr">
+        <is>
+          <t>188.976</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>188.977</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>188.992</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>189.012</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>189.014</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>189.051</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>189.068</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="inlineStr">
+        <is>
+          <t>189.075</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: extend Validation_vs_Melanie sheet with all MS variants
</commit_message>
<xml_diff>
--- a/outputs/scoring_ms_assessment.xlsx
+++ b/outputs/scoring_ms_assessment.xlsx
@@ -23415,7 +23415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23426,82 +23426,37 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_pred</t>
+          <t>Melanie_label</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Our_pred</t>
+          <t>MS original</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_Unpleasant</t>
+          <t>MS Z-Score</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_warm</t>
+          <t>MS Warm rescale</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_green</t>
+          <t>MS Warm+Z-Score</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_floral</t>
+          <t>MS TF-IDF</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_citrus</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Melanie_exotic</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Melanie_Outlayer</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_Unpleasant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_warm</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_green</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_floral</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_citrus</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_exotic</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Ours_Outlayer</t>
+          <t>MS Rohstoffe</t>
         </is>
       </c>
     </row>
@@ -23518,50 +23473,33 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>warm</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>26.513</v>
-      </c>
-      <c r="E2" t="n">
-        <v>69.877</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12.788</v>
-      </c>
-      <c r="G2" t="n">
-        <v>4.324</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5.994</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8.487</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3.058</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1.2564</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1.6261</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.8045</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.1349</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.3794</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.4469</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0057</v>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>unpleasant ✗</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>unpleasant ✗</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>unpleasant ✗</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -23577,50 +23515,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>75.684</v>
-      </c>
-      <c r="E3" t="n">
-        <v>16.019</v>
-      </c>
-      <c r="F3" t="n">
-        <v>38.284</v>
-      </c>
-      <c r="G3" t="n">
-        <v>12.276</v>
-      </c>
-      <c r="H3" t="n">
-        <v>8.273</v>
-      </c>
-      <c r="I3" t="n">
-        <v>8.285</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.8622</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.3231</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.3919</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.0567</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.2056</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.2057</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -23636,50 +23557,33 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>warm</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>21.943</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="F4" t="n">
-        <v>35.943</v>
-      </c>
-      <c r="G4" t="n">
-        <v>12.246</v>
-      </c>
-      <c r="H4" t="n">
-        <v>6.42</v>
-      </c>
-      <c r="I4" t="n">
-        <v>7.907</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.6563</v>
-      </c>
-      <c r="L4" t="n">
-        <v>3.2895</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1.8703</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.9219000000000001</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.6257</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.666</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -23695,50 +23599,33 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>warm</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>11.901</v>
-      </c>
-      <c r="E5" t="n">
-        <v>22.836</v>
-      </c>
-      <c r="F5" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>8.02</v>
-      </c>
-      <c r="H5" t="n">
-        <v>4.055</v>
-      </c>
-      <c r="I5" t="n">
-        <v>4.055</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1.494</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.7286</v>
-      </c>
-      <c r="L5" t="n">
-        <v>1.1302</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.7055</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.2767</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.3038</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.3038</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>unpleasant ✗</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -23754,50 +23641,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>warm</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>4.896</v>
-      </c>
-      <c r="E6" t="n">
-        <v>56.176</v>
-      </c>
-      <c r="F6" t="n">
-        <v>16.324</v>
-      </c>
-      <c r="G6" t="n">
-        <v>75.005</v>
-      </c>
-      <c r="H6" t="n">
-        <v>4.878</v>
-      </c>
-      <c r="I6" t="n">
-        <v>4.878</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.3098</v>
-      </c>
-      <c r="L6" t="n">
-        <v>3.4712</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1.0123</v>
-      </c>
-      <c r="N6" t="n">
-        <v>1.5231</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.3097</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.3097</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>floral ✓</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>floral ✓</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>warm ✗</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>green ✗</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Z-Score CAS alias resolution for ingredient variants (Halal/Kosher)
When an ingredient appears in the recipe CSV under a different CAS registration
than in Melanie's reference data (e.g. Cycloten 80-71-7 vs 765-70-8 Kosher),
load_avg_meli now builds a name-based alias mapping so the correct AvgMeli is used.

- Added _normalize_name() to strip certification qualifiers (Halal, Kosher, natürlich)
- load_avg_meli(csv_path=...) extends the AvgMeli Series with name-matched aliases
- Fixed 80-71-7 (Cycloten) → 765-70-8 AvgMeli: recipe 188.977 warm score now
  matches Melanie's exactly (69.877), prediction flips from Unpleasant → warm
- Updated notebook: interpretation cell documents alias fix and validation results
</commit_message>
<xml_diff>
--- a/outputs/scoring_ms_assessment.xlsx
+++ b/outputs/scoring_ms_assessment.xlsx
@@ -4192,13 +4192,13 @@
         <v>60</v>
       </c>
       <c r="E2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F2" t="n">
         <v>24</v>
       </c>
       <c r="G2" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H2" t="n">
         <v>15</v>
@@ -4500,13 +4500,13 @@
         <v>40</v>
       </c>
       <c r="E13" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F13" t="n">
         <v>31</v>
       </c>
       <c r="G13" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H13" t="n">
         <v>19</v>
@@ -4528,13 +4528,13 @@
         <v>40</v>
       </c>
       <c r="E14" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F14" t="n">
         <v>44</v>
       </c>
       <c r="G14" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" t="n">
         <v>23</v>
@@ -4652,12 +4652,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -4669,12 +4669,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -6624,12 +6624,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -6726,12 +6726,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -14913,7 +14913,7 @@
         <v>73.59229999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>11.552</v>
+        <v>21.5054</v>
       </c>
       <c r="D2" t="n">
         <v>43.503</v>
@@ -14941,7 +14941,7 @@
         <v>4.9448</v>
       </c>
       <c r="C3" t="n">
-        <v>3.4145</v>
+        <v>5.9856</v>
       </c>
       <c r="D3" t="n">
         <v>3.6596</v>
@@ -14969,7 +14969,7 @@
         <v>4.9433</v>
       </c>
       <c r="C4" t="n">
-        <v>3.6397</v>
+        <v>6.2099</v>
       </c>
       <c r="D4" t="n">
         <v>3.6585</v>
@@ -15389,7 +15389,7 @@
         <v>0.7672</v>
       </c>
       <c r="C19" t="n">
-        <v>1.4726</v>
+        <v>2.4394</v>
       </c>
       <c r="D19" t="n">
         <v>7.6868</v>
@@ -15865,7 +15865,7 @@
         <v>97.0471</v>
       </c>
       <c r="C36" t="n">
-        <v>13.4533</v>
+        <v>16.6769</v>
       </c>
       <c r="D36" t="n">
         <v>14.568</v>
@@ -16285,7 +16285,7 @@
         <v>18.6571</v>
       </c>
       <c r="C51" t="n">
-        <v>45.626</v>
+        <v>49.3111</v>
       </c>
       <c r="D51" t="n">
         <v>28.7457</v>
@@ -18189,7 +18189,7 @@
         <v>4.9433</v>
       </c>
       <c r="C119" t="n">
-        <v>3.6397</v>
+        <v>6.2099</v>
       </c>
       <c r="D119" t="n">
         <v>3.6585</v>
@@ -18357,7 +18357,7 @@
         <v>36.8084</v>
       </c>
       <c r="C125" t="n">
-        <v>28.9088</v>
+        <v>69.87690000000001</v>
       </c>
       <c r="D125" t="n">
         <v>12.7875</v>
@@ -18649,7 +18649,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -18664,7 +18664,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -18686,7 +18686,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -18701,7 +18701,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -22941,7 +22941,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -22956,7 +22956,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -23163,7 +23163,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -23178,7 +23178,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>warm</t>
         </is>
       </c>
     </row>
@@ -23415,7 +23415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23426,37 +23426,82 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Melanie_label</t>
+          <t>Melanie_pred</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>MS original</t>
+          <t>Our_pred</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>MS Z-Score</t>
+          <t>Melanie_Unpleasant</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>MS Warm rescale</t>
+          <t>Melanie_warm</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>MS Warm+Z-Score</t>
+          <t>Melanie_green</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>MS TF-IDF</t>
+          <t>Melanie_floral</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>MS Rohstoffe</t>
+          <t>Melanie_citrus</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Melanie_exotic</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Melanie_Outlayer</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_Unpleasant</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_warm</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_green</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_floral</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_citrus</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_exotic</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Ours_Outlayer</t>
         </is>
       </c>
     </row>
@@ -23473,33 +23518,50 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>warm ✓</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>unpleasant ✗</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>unpleasant ✗</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>unpleasant ✗</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>warm ✓</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>26.513</v>
+      </c>
+      <c r="E2" t="n">
+        <v>69.877</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.788</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.324</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5.994</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8.487</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3.058</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.2564</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.6261</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.8045</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1349</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.3794</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.4469</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0057</v>
       </c>
     </row>
     <row r="3">
@@ -23515,33 +23577,50 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>unpleasant ✓</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>unpleasant ✓</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>unpleasant ✓</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>unpleasant ✓</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>unpleasant ✓</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>unpleasant ✓</t>
-        </is>
+          <t>Unpleasant</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>75.684</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16.019</v>
+      </c>
+      <c r="F3" t="n">
+        <v>38.284</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12.276</v>
+      </c>
+      <c r="H3" t="n">
+        <v>8.273</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8.285</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.8622</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.3231</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3919</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.0567</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.2056</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.2057</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -23557,33 +23636,50 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>21.943</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F4" t="n">
+        <v>35.943</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12.246</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7.907</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.6563</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3.2895</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1.8703</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.9219000000000001</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.6257</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -23599,33 +23695,50 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>unpleasant ✗</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>11.901</v>
+      </c>
+      <c r="E5" t="n">
+        <v>22.836</v>
+      </c>
+      <c r="F5" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.055</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.055</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.494</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.7286</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.1302</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.7055</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.2767</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.3038</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.3038</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -23641,33 +23754,50 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>floral ✓</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>floral ✓</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>warm ✗</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>green ✗</t>
-        </is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.896</v>
+      </c>
+      <c r="E6" t="n">
+        <v>56.176</v>
+      </c>
+      <c r="F6" t="n">
+        <v>16.324</v>
+      </c>
+      <c r="G6" t="n">
+        <v>75.005</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4.878</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.878</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3098</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3.4712</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.0123</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1.5231</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.3097</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.3097</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: remove exotic→dairy and Outlayer→Walderdbeere MS cluster mappings
exotic and Outlayer are distinct MS clusters with no panel equivalent.
Mapping them to dairy/Walderdbeere was incorrect. Both are now excluded
from the panel accuracy comparison (MS_TO_PANEL reduced to 5 entries).
Accuracy numbers unchanged since neither exotic nor Outlayer was ever
predicted for the 10 confident GT recipes.
</commit_message>
<xml_diff>
--- a/outputs/scoring_ms_assessment.xlsx
+++ b/outputs/scoring_ms_assessment.xlsx
@@ -5607,11 +5607,7 @@
           <t>exotic</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -5896,11 +5892,7 @@
           <t>exotic</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
+      <c r="C76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -8376,11 +8368,6 @@
           <t>exotic</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
       <c r="D59" t="n">
         <v>0.4559</v>
       </c>
@@ -8816,11 +8803,6 @@
       <c r="B76" t="inlineStr">
         <is>
           <t>exotic</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>dairy</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -20724,19 +20706,9 @@
           <t>exotic</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>green</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>dairy</t>
         </is>
       </c>
     </row>
@@ -21353,19 +21325,9 @@
           <t>exotic</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
       <c r="F76" t="inlineStr">
         <is>
           <t>warm</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>dairy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add GT_panel column to ZScore prediction sheets
GT_panel contains the panel ground truth for the 10 Verkostung recipes
(empty for all others), making it possible to directly compare
ZScore_panel_name against what the panel actually decided.
</commit_message>
<xml_diff>
--- a/outputs/scoring_ms_assessment.xlsx
+++ b/outputs/scoring_ms_assessment.xlsx
@@ -6840,7 +6840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6899,6 +6899,11 @@
           <t>in_verkostung</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>GT_panel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -6940,6 +6945,11 @@
       <c r="K2" t="b">
         <v>1</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -6981,6 +6991,7 @@
       <c r="K3" t="b">
         <v>0</v>
       </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -7022,6 +7033,7 @@
       <c r="K4" t="b">
         <v>0</v>
       </c>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -7063,6 +7075,7 @@
       <c r="K5" t="b">
         <v>0</v>
       </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -7104,6 +7117,11 @@
       <c r="K6" t="b">
         <v>1</v>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -7145,6 +7163,7 @@
       <c r="K7" t="b">
         <v>0</v>
       </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -7186,6 +7205,7 @@
       <c r="K8" t="b">
         <v>0</v>
       </c>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -7227,6 +7247,7 @@
       <c r="K9" t="b">
         <v>0</v>
       </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -7268,6 +7289,11 @@
       <c r="K10" t="b">
         <v>1</v>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -7309,6 +7335,7 @@
       <c r="K11" t="b">
         <v>0</v>
       </c>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -7350,6 +7377,7 @@
       <c r="K12" t="b">
         <v>0</v>
       </c>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -7391,6 +7419,7 @@
       <c r="K13" t="b">
         <v>0</v>
       </c>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -7432,6 +7461,7 @@
       <c r="K14" t="b">
         <v>0</v>
       </c>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -7473,6 +7503,7 @@
       <c r="K15" t="b">
         <v>0</v>
       </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -7514,6 +7545,7 @@
       <c r="K16" t="b">
         <v>0</v>
       </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -7555,6 +7587,7 @@
       <c r="K17" t="b">
         <v>0</v>
       </c>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -7596,6 +7629,7 @@
       <c r="K18" t="b">
         <v>0</v>
       </c>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -7636,6 +7670,11 @@
       </c>
       <c r="K19" t="b">
         <v>1</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -7674,6 +7713,7 @@
       <c r="K20" t="b">
         <v>0</v>
       </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -7711,6 +7751,7 @@
       <c r="K21" t="b">
         <v>0</v>
       </c>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -7752,6 +7793,7 @@
       <c r="K22" t="b">
         <v>0</v>
       </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -7793,6 +7835,7 @@
       <c r="K23" t="b">
         <v>0</v>
       </c>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -7834,6 +7877,7 @@
       <c r="K24" t="b">
         <v>0</v>
       </c>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -7875,6 +7919,7 @@
       <c r="K25" t="b">
         <v>0</v>
       </c>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -7916,6 +7961,11 @@
       <c r="K26" t="b">
         <v>1</v>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -7957,6 +8007,7 @@
       <c r="K27" t="b">
         <v>0</v>
       </c>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -7998,6 +8049,7 @@
       <c r="K28" t="b">
         <v>0</v>
       </c>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -8039,6 +8091,7 @@
       <c r="K29" t="b">
         <v>0</v>
       </c>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -8080,6 +8133,7 @@
       <c r="K30" t="b">
         <v>0</v>
       </c>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -8121,6 +8175,7 @@
       <c r="K31" t="b">
         <v>0</v>
       </c>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -8162,6 +8217,7 @@
       <c r="K32" t="b">
         <v>0</v>
       </c>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -8203,6 +8259,7 @@
       <c r="K33" t="b">
         <v>0</v>
       </c>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -8244,6 +8301,7 @@
       <c r="K34" t="b">
         <v>0</v>
       </c>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -8285,6 +8343,7 @@
       <c r="K35" t="b">
         <v>0</v>
       </c>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -8326,6 +8385,7 @@
       <c r="K36" t="b">
         <v>0</v>
       </c>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -8367,6 +8427,7 @@
       <c r="K37" t="b">
         <v>0</v>
       </c>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -8408,6 +8469,7 @@
       <c r="K38" t="b">
         <v>0</v>
       </c>
+      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -8449,6 +8511,7 @@
       <c r="K39" t="b">
         <v>0</v>
       </c>
+      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -8490,6 +8553,7 @@
       <c r="K40" t="b">
         <v>0</v>
       </c>
+      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
@@ -8531,6 +8595,7 @@
       <c r="K41" t="b">
         <v>0</v>
       </c>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -8572,6 +8637,7 @@
       <c r="K42" t="b">
         <v>0</v>
       </c>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
@@ -8613,6 +8679,7 @@
       <c r="K43" t="b">
         <v>0</v>
       </c>
+      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -8654,6 +8721,7 @@
       <c r="K44" t="b">
         <v>0</v>
       </c>
+      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -8695,6 +8763,7 @@
       <c r="K45" t="b">
         <v>0</v>
       </c>
+      <c r="L45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
@@ -8736,6 +8805,7 @@
       <c r="K46" t="b">
         <v>0</v>
       </c>
+      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
@@ -8777,6 +8847,7 @@
       <c r="K47" t="b">
         <v>0</v>
       </c>
+      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
@@ -8818,6 +8889,7 @@
       <c r="K48" t="b">
         <v>0</v>
       </c>
+      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -8859,6 +8931,7 @@
       <c r="K49" t="b">
         <v>0</v>
       </c>
+      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
@@ -8900,6 +8973,7 @@
       <c r="K50" t="b">
         <v>0</v>
       </c>
+      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
@@ -8941,6 +9015,7 @@
       <c r="K51" t="b">
         <v>0</v>
       </c>
+      <c r="L51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
@@ -8982,6 +9057,7 @@
       <c r="K52" t="b">
         <v>0</v>
       </c>
+      <c r="L52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -9023,6 +9099,7 @@
       <c r="K53" t="b">
         <v>0</v>
       </c>
+      <c r="L53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
@@ -9064,6 +9141,7 @@
       <c r="K54" t="b">
         <v>0</v>
       </c>
+      <c r="L54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
@@ -9105,6 +9183,7 @@
       <c r="K55" t="b">
         <v>0</v>
       </c>
+      <c r="L55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
@@ -9146,6 +9225,7 @@
       <c r="K56" t="b">
         <v>0</v>
       </c>
+      <c r="L56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
@@ -9187,6 +9267,7 @@
       <c r="K57" t="b">
         <v>0</v>
       </c>
+      <c r="L57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
@@ -9228,6 +9309,11 @@
       <c r="K58" t="b">
         <v>1</v>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
@@ -9269,6 +9355,7 @@
       <c r="K59" t="b">
         <v>0</v>
       </c>
+      <c r="L59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -9310,6 +9397,7 @@
       <c r="K60" t="b">
         <v>0</v>
       </c>
+      <c r="L60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
@@ -9351,6 +9439,7 @@
       <c r="K61" t="b">
         <v>0</v>
       </c>
+      <c r="L61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
@@ -9392,6 +9481,7 @@
       <c r="K62" t="b">
         <v>0</v>
       </c>
+      <c r="L62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
@@ -9433,6 +9523,7 @@
       <c r="K63" t="b">
         <v>0</v>
       </c>
+      <c r="L63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
@@ -9474,6 +9565,7 @@
       <c r="K64" t="b">
         <v>0</v>
       </c>
+      <c r="L64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
@@ -9515,6 +9607,7 @@
       <c r="K65" t="b">
         <v>0</v>
       </c>
+      <c r="L65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
@@ -9556,6 +9649,11 @@
       <c r="K66" t="b">
         <v>1</v>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
@@ -9597,6 +9695,7 @@
       <c r="K67" t="b">
         <v>0</v>
       </c>
+      <c r="L67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
@@ -9638,6 +9737,7 @@
       <c r="K68" t="b">
         <v>0</v>
       </c>
+      <c r="L68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
@@ -9679,6 +9779,7 @@
       <c r="K69" t="b">
         <v>0</v>
       </c>
+      <c r="L69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
@@ -9720,6 +9821,7 @@
       <c r="K70" t="b">
         <v>0</v>
       </c>
+      <c r="L70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
@@ -9761,6 +9863,7 @@
       <c r="K71" t="b">
         <v>0</v>
       </c>
+      <c r="L71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
@@ -9802,6 +9905,7 @@
       <c r="K72" t="b">
         <v>0</v>
       </c>
+      <c r="L72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
@@ -9843,6 +9947,11 @@
       <c r="K73" t="b">
         <v>1</v>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
@@ -9884,6 +9993,7 @@
       <c r="K74" t="b">
         <v>0</v>
       </c>
+      <c r="L74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
@@ -9925,6 +10035,7 @@
       <c r="K75" t="b">
         <v>0</v>
       </c>
+      <c r="L75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
@@ -9966,6 +10077,7 @@
       <c r="K76" t="b">
         <v>0</v>
       </c>
+      <c r="L76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -10007,6 +10119,7 @@
       <c r="K77" t="b">
         <v>0</v>
       </c>
+      <c r="L77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
@@ -10048,6 +10161,7 @@
       <c r="K78" t="b">
         <v>0</v>
       </c>
+      <c r="L78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
@@ -10089,6 +10203,7 @@
       <c r="K79" t="b">
         <v>0</v>
       </c>
+      <c r="L79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
@@ -10130,6 +10245,7 @@
       <c r="K80" t="b">
         <v>0</v>
       </c>
+      <c r="L80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
@@ -10171,6 +10287,7 @@
       <c r="K81" t="b">
         <v>0</v>
       </c>
+      <c r="L81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
@@ -10212,6 +10329,7 @@
       <c r="K82" t="b">
         <v>0</v>
       </c>
+      <c r="L82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
@@ -10253,6 +10371,7 @@
       <c r="K83" t="b">
         <v>0</v>
       </c>
+      <c r="L83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
@@ -10294,6 +10413,7 @@
       <c r="K84" t="b">
         <v>0</v>
       </c>
+      <c r="L84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
@@ -10335,6 +10455,7 @@
       <c r="K85" t="b">
         <v>0</v>
       </c>
+      <c r="L85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
@@ -10376,6 +10497,7 @@
       <c r="K86" t="b">
         <v>0</v>
       </c>
+      <c r="L86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
@@ -10417,6 +10539,7 @@
       <c r="K87" t="b">
         <v>0</v>
       </c>
+      <c r="L87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
@@ -10458,6 +10581,7 @@
       <c r="K88" t="b">
         <v>0</v>
       </c>
+      <c r="L88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
@@ -10499,6 +10623,7 @@
       <c r="K89" t="b">
         <v>0</v>
       </c>
+      <c r="L89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
@@ -10540,6 +10665,7 @@
       <c r="K90" t="b">
         <v>0</v>
       </c>
+      <c r="L90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
@@ -10581,6 +10707,7 @@
       <c r="K91" t="b">
         <v>0</v>
       </c>
+      <c r="L91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
@@ -10622,6 +10749,7 @@
       <c r="K92" t="b">
         <v>0</v>
       </c>
+      <c r="L92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
@@ -10663,6 +10791,7 @@
       <c r="K93" t="b">
         <v>0</v>
       </c>
+      <c r="L93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
@@ -10704,6 +10833,7 @@
       <c r="K94" t="b">
         <v>0</v>
       </c>
+      <c r="L94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
@@ -10745,6 +10875,7 @@
       <c r="K95" t="b">
         <v>0</v>
       </c>
+      <c r="L95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
@@ -10786,6 +10917,7 @@
       <c r="K96" t="b">
         <v>0</v>
       </c>
+      <c r="L96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
@@ -10827,6 +10959,7 @@
       <c r="K97" t="b">
         <v>0</v>
       </c>
+      <c r="L97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
@@ -10868,6 +11001,11 @@
       <c r="K98" t="b">
         <v>1</v>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
@@ -10909,6 +11047,7 @@
       <c r="K99" t="b">
         <v>0</v>
       </c>
+      <c r="L99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
@@ -10950,6 +11089,11 @@
       <c r="K100" t="b">
         <v>1</v>
       </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
@@ -10991,6 +11135,7 @@
       <c r="K101" t="b">
         <v>0</v>
       </c>
+      <c r="L101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
@@ -11032,6 +11177,7 @@
       <c r="K102" t="b">
         <v>0</v>
       </c>
+      <c r="L102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
@@ -11073,6 +11219,7 @@
       <c r="K103" t="b">
         <v>0</v>
       </c>
+      <c r="L103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
@@ -11114,6 +11261,7 @@
       <c r="K104" t="b">
         <v>0</v>
       </c>
+      <c r="L104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
@@ -11155,6 +11303,7 @@
       <c r="K105" t="b">
         <v>0</v>
       </c>
+      <c r="L105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
@@ -11196,6 +11345,7 @@
       <c r="K106" t="b">
         <v>0</v>
       </c>
+      <c r="L106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
@@ -11237,6 +11387,7 @@
       <c r="K107" t="b">
         <v>0</v>
       </c>
+      <c r="L107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
@@ -11278,6 +11429,7 @@
       <c r="K108" t="b">
         <v>0</v>
       </c>
+      <c r="L108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
@@ -11319,6 +11471,7 @@
       <c r="K109" t="b">
         <v>0</v>
       </c>
+      <c r="L109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
@@ -11360,6 +11513,7 @@
       <c r="K110" t="b">
         <v>0</v>
       </c>
+      <c r="L110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
@@ -11401,6 +11555,7 @@
       <c r="K111" t="b">
         <v>0</v>
       </c>
+      <c r="L111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
@@ -11442,6 +11597,7 @@
       <c r="K112" t="b">
         <v>0</v>
       </c>
+      <c r="L112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
@@ -11483,6 +11639,7 @@
       <c r="K113" t="b">
         <v>0</v>
       </c>
+      <c r="L113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
@@ -11524,6 +11681,7 @@
       <c r="K114" t="b">
         <v>0</v>
       </c>
+      <c r="L114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
@@ -11565,6 +11723,7 @@
       <c r="K115" t="b">
         <v>0</v>
       </c>
+      <c r="L115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
@@ -11606,6 +11765,7 @@
       <c r="K116" t="b">
         <v>0</v>
       </c>
+      <c r="L116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
@@ -11647,6 +11807,7 @@
       <c r="K117" t="b">
         <v>0</v>
       </c>
+      <c r="L117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
@@ -11688,6 +11849,7 @@
       <c r="K118" t="b">
         <v>0</v>
       </c>
+      <c r="L118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
@@ -11729,6 +11891,7 @@
       <c r="K119" t="b">
         <v>0</v>
       </c>
+      <c r="L119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
@@ -11770,6 +11933,7 @@
       <c r="K120" t="b">
         <v>0</v>
       </c>
+      <c r="L120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
@@ -11811,6 +11975,7 @@
       <c r="K121" t="b">
         <v>0</v>
       </c>
+      <c r="L121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
@@ -11852,6 +12017,7 @@
       <c r="K122" t="b">
         <v>0</v>
       </c>
+      <c r="L122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
@@ -11893,6 +12059,7 @@
       <c r="K123" t="b">
         <v>0</v>
       </c>
+      <c r="L123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
@@ -11934,6 +12101,7 @@
       <c r="K124" t="b">
         <v>0</v>
       </c>
+      <c r="L124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
@@ -11975,6 +12143,7 @@
       <c r="K125" t="b">
         <v>0</v>
       </c>
+      <c r="L125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
@@ -12016,6 +12185,7 @@
       <c r="K126" t="b">
         <v>0</v>
       </c>
+      <c r="L126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
@@ -12057,6 +12227,7 @@
       <c r="K127" t="b">
         <v>0</v>
       </c>
+      <c r="L127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
@@ -12098,6 +12269,7 @@
       <c r="K128" t="b">
         <v>0</v>
       </c>
+      <c r="L128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
@@ -12139,6 +12311,7 @@
       <c r="K129" t="b">
         <v>0</v>
       </c>
+      <c r="L129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
@@ -12180,6 +12353,7 @@
       <c r="K130" t="b">
         <v>0</v>
       </c>
+      <c r="L130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
@@ -12221,6 +12395,7 @@
       <c r="K131" t="b">
         <v>0</v>
       </c>
+      <c r="L131" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12233,7 +12408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12254,6 +12429,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>GT_panel</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>in_verkostung</t>
         </is>
       </c>
@@ -12274,7 +12454,12 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D2" t="b">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12294,7 +12479,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D3" t="b">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12314,7 +12500,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D4" t="b">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12334,7 +12521,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D5" t="b">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12354,7 +12542,12 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D6" t="b">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12374,7 +12567,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D7" t="b">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12394,7 +12588,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D8" t="b">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12414,7 +12609,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D9" t="b">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12434,7 +12630,12 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D10" t="b">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12454,7 +12655,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D11" t="b">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12474,7 +12676,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D12" t="b">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12494,7 +12697,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D13" t="b">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12514,7 +12718,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D14" t="b">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12534,7 +12739,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D15" t="b">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12554,7 +12760,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D16" t="b">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12574,7 +12781,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D17" t="b">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12594,7 +12802,8 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D18" t="b">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12614,7 +12823,12 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="D19" t="b">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12630,7 +12844,8 @@
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="b">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12646,7 +12861,8 @@
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="b">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12666,7 +12882,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D22" t="b">
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12686,7 +12903,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D23" t="b">
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12706,7 +12924,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D24" t="b">
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12726,7 +12945,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D25" t="b">
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12746,7 +12966,12 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D26" t="b">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12766,7 +12991,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D27" t="b">
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12786,7 +13012,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D28" t="b">
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12806,7 +13033,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D29" t="b">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12826,7 +13054,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D30" t="b">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12846,7 +13075,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D31" t="b">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12866,7 +13096,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D32" t="b">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12886,7 +13117,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D33" t="b">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12906,7 +13138,8 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="D34" t="b">
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12926,7 +13159,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D35" t="b">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12946,7 +13180,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D36" t="b">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12966,7 +13201,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D37" t="b">
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12986,7 +13222,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D38" t="b">
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13006,7 +13243,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D39" t="b">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13026,7 +13264,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D40" t="b">
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13046,7 +13285,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D41" t="b">
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13066,7 +13306,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D42" t="b">
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13086,7 +13327,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D43" t="b">
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13106,7 +13348,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D44" t="b">
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13126,7 +13369,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D45" t="b">
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13146,7 +13390,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D46" t="b">
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13166,7 +13411,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D47" t="b">
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13186,7 +13432,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D48" t="b">
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13206,7 +13453,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D49" t="b">
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13226,7 +13474,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D50" t="b">
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13246,7 +13495,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D51" t="b">
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13266,7 +13516,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D52" t="b">
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13286,7 +13537,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D53" t="b">
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13306,7 +13558,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D54" t="b">
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13326,7 +13579,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D55" t="b">
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13346,7 +13600,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D56" t="b">
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13366,7 +13621,8 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D57" t="b">
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13386,7 +13642,12 @@
           <t>green</t>
         </is>
       </c>
-      <c r="D58" t="b">
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="E58" t="b">
         <v>1</v>
       </c>
     </row>
@@ -13406,7 +13667,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D59" t="b">
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13426,7 +13688,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D60" t="b">
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13446,7 +13709,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D61" t="b">
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13466,7 +13730,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D62" t="b">
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13486,7 +13751,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D63" t="b">
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13506,7 +13772,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D64" t="b">
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13526,7 +13793,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D65" t="b">
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13546,7 +13814,12 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D66" t="b">
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="E66" t="b">
         <v>1</v>
       </c>
     </row>
@@ -13566,7 +13839,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D67" t="b">
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13586,7 +13860,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D68" t="b">
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13606,7 +13881,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D69" t="b">
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13626,7 +13902,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D70" t="b">
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13646,7 +13923,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D71" t="b">
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13666,7 +13944,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D72" t="b">
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13686,7 +13965,12 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D73" t="b">
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E73" t="b">
         <v>1</v>
       </c>
     </row>
@@ -13706,7 +13990,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D74" t="b">
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13726,7 +14011,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D75" t="b">
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13746,7 +14032,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D76" t="b">
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13766,7 +14053,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D77" t="b">
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13786,7 +14074,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D78" t="b">
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13806,7 +14095,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D79" t="b">
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13826,7 +14116,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D80" t="b">
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13846,7 +14137,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D81" t="b">
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13866,7 +14158,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D82" t="b">
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13886,7 +14179,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D83" t="b">
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13906,7 +14200,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D84" t="b">
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13926,7 +14221,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D85" t="b">
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13946,7 +14242,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D86" t="b">
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13966,7 +14263,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D87" t="b">
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="b">
         <v>0</v>
       </c>
     </row>
@@ -13986,7 +14284,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D88" t="b">
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14006,7 +14305,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D89" t="b">
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14026,7 +14326,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D90" t="b">
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14046,7 +14347,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D91" t="b">
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14066,7 +14368,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D92" t="b">
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14086,7 +14389,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D93" t="b">
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14106,7 +14410,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D94" t="b">
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14126,7 +14431,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D95" t="b">
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14146,7 +14452,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D96" t="b">
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14166,7 +14473,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D97" t="b">
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14186,7 +14494,12 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D98" t="b">
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="E98" t="b">
         <v>1</v>
       </c>
     </row>
@@ -14206,7 +14519,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D99" t="b">
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14226,7 +14540,12 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D100" t="b">
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E100" t="b">
         <v>1</v>
       </c>
     </row>
@@ -14246,7 +14565,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D101" t="b">
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14266,7 +14586,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D102" t="b">
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14286,7 +14607,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D103" t="b">
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14306,7 +14628,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D104" t="b">
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14326,7 +14649,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D105" t="b">
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14346,7 +14670,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D106" t="b">
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14366,7 +14691,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D107" t="b">
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14386,7 +14712,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D108" t="b">
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14406,7 +14733,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D109" t="b">
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14426,7 +14754,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D110" t="b">
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14446,7 +14775,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D111" t="b">
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14466,7 +14796,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D112" t="b">
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14486,7 +14817,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D113" t="b">
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14506,7 +14838,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D114" t="b">
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14526,7 +14859,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D115" t="b">
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14546,7 +14880,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D116" t="b">
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14566,7 +14901,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D117" t="b">
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14586,7 +14922,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D118" t="b">
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14606,7 +14943,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D119" t="b">
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14626,7 +14964,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D120" t="b">
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14646,7 +14985,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D121" t="b">
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14666,7 +15006,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D122" t="b">
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14686,7 +15027,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D123" t="b">
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14706,7 +15048,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D124" t="b">
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14726,7 +15069,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D125" t="b">
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14746,7 +15090,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D126" t="b">
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14766,7 +15111,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D127" t="b">
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14786,7 +15132,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D128" t="b">
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14806,7 +15153,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D129" t="b">
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14826,7 +15174,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D130" t="b">
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="b">
         <v>0</v>
       </c>
     </row>
@@ -14846,7 +15195,8 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="D131" t="b">
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>